<commit_message>
version2: sync outputs + remove cv_r2_summary
- Drop cv_r2_summary pipeline and table
- Regenerated plots/tables/reports
- Docs aligned with tuning-only CV artifacts

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/outputs/eda/tables/00_data_audit.xlsx
+++ b/outputs/eda/tables/00_data_audit.xlsx
@@ -484,31 +484,31 @@
         <v>0</v>
       </c>
       <c r="D2">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="E2">
         <v>0</v>
       </c>
       <c r="F2">
-        <v>100</v>
+        <v>18</v>
       </c>
       <c r="G2">
-        <v>5.196078431372549</v>
+        <v>3.214285714285714</v>
       </c>
       <c r="H2">
-        <v>16.57501687220033</v>
+        <v>5.32683441033836</v>
       </c>
       <c r="I2">
-        <v>0</v>
+        <v>1.05</v>
       </c>
       <c r="J2">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="K2">
-        <v>0.75</v>
+        <v>2.85</v>
       </c>
       <c r="L2">
-        <v>0.75</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="3" spans="1:12">
@@ -522,31 +522,31 @@
         <v>0</v>
       </c>
       <c r="D3">
-        <v>42</v>
+        <v>14</v>
       </c>
       <c r="E3">
         <v>7.6</v>
       </c>
       <c r="F3">
-        <v>739.2</v>
+        <v>150</v>
       </c>
       <c r="G3">
-        <v>136.8298039215686</v>
+        <v>43.50000000000001</v>
       </c>
       <c r="H3">
-        <v>136.859404784475</v>
+        <v>42.57419659118203</v>
       </c>
       <c r="I3">
-        <v>100</v>
+        <v>35.75</v>
       </c>
       <c r="J3">
-        <v>36.85</v>
+        <v>13.925</v>
       </c>
       <c r="K3">
-        <v>223.4</v>
+        <v>39.375</v>
       </c>
       <c r="L3">
-        <v>186.55</v>
+        <v>25.45</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -560,31 +560,31 @@
         <v>0</v>
       </c>
       <c r="D4">
-        <v>42</v>
+        <v>14</v>
       </c>
       <c r="E4">
-        <v>24</v>
+        <v>32.7</v>
       </c>
       <c r="F4">
-        <v>85</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="G4">
-        <v>60.01764705882353</v>
+        <v>67.4357142857143</v>
       </c>
       <c r="H4">
-        <v>15.43044660251093</v>
+        <v>13.0981858487148</v>
       </c>
       <c r="I4">
-        <v>64</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="J4">
-        <v>50.1</v>
+        <v>64.7</v>
       </c>
       <c r="K4">
-        <v>72</v>
+        <v>74.75</v>
       </c>
       <c r="L4">
-        <v>21.9</v>
+        <v>10.05</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -598,31 +598,31 @@
         <v>0</v>
       </c>
       <c r="D5">
-        <v>47</v>
+        <v>14</v>
       </c>
       <c r="E5">
-        <v>13.9</v>
+        <v>123.4</v>
       </c>
       <c r="F5">
-        <v>552</v>
+        <v>318.1</v>
       </c>
       <c r="G5">
-        <v>249.9470588235294</v>
+        <v>262.9642857142857</v>
       </c>
       <c r="H5">
-        <v>99.22875662415846</v>
+        <v>50.1360396573909</v>
       </c>
       <c r="I5">
-        <v>270</v>
+        <v>273.5</v>
       </c>
       <c r="J5">
-        <v>193.9</v>
+        <v>260.225</v>
       </c>
       <c r="K5">
-        <v>305</v>
+        <v>291.25</v>
       </c>
       <c r="L5">
-        <v>111.1</v>
+        <v>31.02499999999998</v>
       </c>
     </row>
     <row r="6" spans="1:12">
@@ -636,31 +636,31 @@
         <v>0</v>
       </c>
       <c r="D6">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="E6">
         <v>27</v>
       </c>
       <c r="F6">
-        <v>98.5</v>
+        <v>97</v>
       </c>
       <c r="G6">
-        <v>77.49019607843137</v>
+        <v>75.70714285714287</v>
       </c>
       <c r="H6">
-        <v>17.16407008727197</v>
+        <v>22.12560174881697</v>
       </c>
       <c r="I6">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J6">
-        <v>70</v>
+        <v>77.25</v>
       </c>
       <c r="K6">
-        <v>90.34999999999999</v>
+        <v>92</v>
       </c>
       <c r="L6">
-        <v>20.34999999999999</v>
+        <v>14.75</v>
       </c>
     </row>
   </sheetData>
@@ -670,7 +670,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
@@ -689,10 +689,10 @@
         <v>0</v>
       </c>
       <c r="B2">
-        <v>36</v>
+        <v>4</v>
       </c>
       <c r="C2">
-        <v>0.7058823529411765</v>
+        <v>0.2857142857142857</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -703,7 +703,7 @@
         <v>1</v>
       </c>
       <c r="C3">
-        <v>0.0196078431372549</v>
+        <v>0.07142857142857142</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -714,7 +714,7 @@
         <v>1</v>
       </c>
       <c r="C4">
-        <v>0.0196078431372549</v>
+        <v>0.07142857142857142</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -725,7 +725,7 @@
         <v>1</v>
       </c>
       <c r="C5">
-        <v>0.0196078431372549</v>
+        <v>0.07142857142857142</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -736,7 +736,7 @@
         <v>1</v>
       </c>
       <c r="C6">
-        <v>0.0196078431372549</v>
+        <v>0.07142857142857142</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -747,7 +747,7 @@
         <v>1</v>
       </c>
       <c r="C7">
-        <v>0.0196078431372549</v>
+        <v>0.07142857142857142</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -758,7 +758,7 @@
         <v>1</v>
       </c>
       <c r="C8">
-        <v>0.0196078431372549</v>
+        <v>0.07142857142857142</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -769,7 +769,7 @@
         <v>1</v>
       </c>
       <c r="C9">
-        <v>0.0196078431372549</v>
+        <v>0.07142857142857142</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -780,84 +780,29 @@
         <v>1</v>
       </c>
       <c r="C10">
-        <v>0.0196078431372549</v>
+        <v>0.07142857142857142</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B11">
         <v>1</v>
       </c>
       <c r="C11">
-        <v>0.0196078431372549</v>
+        <v>0.07142857142857142</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="B12">
         <v>1</v>
       </c>
       <c r="C12">
-        <v>0.0196078431372549</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3">
-      <c r="A13">
-        <v>18</v>
-      </c>
-      <c r="B13">
-        <v>1</v>
-      </c>
-      <c r="C13">
-        <v>0.0196078431372549</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3">
-      <c r="A14">
-        <v>20</v>
-      </c>
-      <c r="B14">
-        <v>1</v>
-      </c>
-      <c r="C14">
-        <v>0.0196078431372549</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3">
-      <c r="A15">
-        <v>40</v>
-      </c>
-      <c r="B15">
-        <v>1</v>
-      </c>
-      <c r="C15">
-        <v>0.0196078431372549</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3">
-      <c r="A16">
-        <v>50</v>
-      </c>
-      <c r="B16">
-        <v>1</v>
-      </c>
-      <c r="C16">
-        <v>0.0196078431372549</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3">
-      <c r="A17">
-        <v>100</v>
-      </c>
-      <c r="B17">
-        <v>1</v>
-      </c>
-      <c r="C17">
-        <v>0.0196078431372549</v>
+        <v>0.07142857142857142</v>
       </c>
     </row>
   </sheetData>

</xml_diff>